<commit_message>
Update dataset: hi-hindustani-rag (25 records)
</commit_message>
<xml_diff>
--- a/music/hi-hindustani-rag_HI.xlsx
+++ b/music/hi-hindustani-rag_HI.xlsx
@@ -11,189 +11,240 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="78">
   <si>
     <t>नाम</t>
   </si>
   <si>
-    <t>अंग्रेज़ी नाम</t>
-  </si>
-  <si>
-    <t>स्रोत का अंग्रेज़ी विवरण</t>
-  </si>
-  <si>
-    <t>वर्गीकरण</t>
+    <t>मूल विवरण</t>
   </si>
   <si>
     <t>स्रोत लिंक</t>
   </si>
   <si>
-    <t>भैरव</t>
-  </si>
-  <si>
-    <t>Bhairav</t>
-  </si>
-  <si>
-    <t>Hindustani raga</t>
-  </si>
-  <si>
-    <t>राग</t>
-  </si>
-  <si>
-    <t>https://www.wikidata.org/wiki/Q2321739</t>
+    <t>अल्हैयाबिलावल</t>
+  </si>
+  <si>
+    <t>यह राग बिलावल थाट से निकलता है। इसमें सब स्वर शुद्ध लगते हैं। केवल अवरोह में थोड़ा कोमल नी लगाया जाता है। आरोह में म वर्ज्य हैं, इसलिये इस राग की जाति षाडव-संपूर्ण मानी जाती है। वादी ध और सम्वादी ग माना जाता है।</t>
+  </si>
+  <si>
+    <t>https://hi.wikipedia.org/w/index.php?title=%E0%A4%85%E0%A4%B2%E0%A5%8D%E0%A4%B9%E0%A5%88%E0%A4%AF%E0%A4%BE%E0%A4%AC%E0%A4%BF%E0%A4%B2%E0%A4%BE%E0%A4%B5%E0%A4%B2&amp;oldid=3972818</t>
+  </si>
+  <si>
+    <t>काफ़ी राग</t>
+  </si>
+  <si>
+    <t>यह राग काफी थाट से निकलता है। इसमें ः?ग"' और ः?नी"' कोमल वाकी सब शुद्ध स्वर लगते हैं। वादी स्वर ः?प"' और सम्वादी ः?स"' माना जाता है। इसकी जाति सम्पूर्ण मानी जाती है। इस राग में होली के गीत बहुत गाये जाते हैं। ठुमरी भी गाई जाती है।</t>
+  </si>
+  <si>
+    <t>https://hi.wikipedia.org/w/index.php?title=%E0%A4%95%E0%A4%BE%E0%A4%AB%E0%A4%BC%E0%A5%80_%E0%A4%B0%E0%A4%BE%E0%A4%97&amp;oldid=6404498</t>
+  </si>
+  <si>
+    <t>जयजयवन्ती</t>
+  </si>
+  <si>
+    <t>जयजयवन्ती , हिन्दुस्तानी शास्त्रीय संगीत का एक राग है। गुरु ग्रन्थ साहिब के अनुसार यह राग, बिलवाल और सोरठ नामक दो अन्य रागों का मिश्रण है। यह राग, गुरबानी के उत्तरार्ध में आया है। नौवें गुरु तेग बहादुर जी ने जयजयवन्ती में ४ पदों की रचना की है।</t>
+  </si>
+  <si>
+    <t>https://hi.wikipedia.org/w/index.php?title=%E0%A4%9C%E0%A4%AF%E0%A4%9C%E0%A4%AF%E0%A4%B5%E0%A4%A8%E0%A5%8D%E0%A4%A4%E0%A5%80&amp;oldid=4564688</t>
+  </si>
+  <si>
+    <t>जौनपुरी</t>
+  </si>
+  <si>
+    <t>जौनपुरी राग को असवारी थाट से उपजा हुआ राग माना गया है। इस राग में ग , ध, नी स्वर कोमल लगते हैं । आरोह में ग (गंधार ) वर्ज्य है अर्थात गाते बजाते समय आरोह में ग स्वर को छोड़ देते हैं। अवरोह में सातों स्वर प्रयोग किये जाते हैं। अतः इस राग की जाती षाडव-संपूर्ण है। जौनपुरी राग का वादी स्वर ध (धैवत )और संवादी स्वर ग (गंधार) है।</t>
+  </si>
+  <si>
+    <t>https://hi.wikipedia.org/w/index.php?title=%E0%A4%9C%E0%A5%8C%E0%A4%A8%E0%A4%AA%E0%A5%81%E0%A4%B0%E0%A5%80&amp;oldid=6021084</t>
+  </si>
+  <si>
+    <t>बिहाग</t>
+  </si>
+  <si>
+    <t>यह राग बिलावल ठाठ से उतपन्न होता है। इसके आरोह में रे और ध नहीं लगाते और अवरोह में सातों स्वर लगते हैं, इसलिये इसकी जाति औडव-सम्पूर्ण मानी जाती है। इसमें सब स्वर शुद्ध लगते है। कुशल संगीतज्ञ बड़ी कुशलता से इस राग में तीव्र म' का भी प्रयोग करते हैं। वादी स्वर ग और संवादी स्वर नी माना जाता है।</t>
+  </si>
+  <si>
+    <t>https://hi.wikipedia.org/w/index.php?title=%E0%A4%AC%E0%A4%BF%E0%A4%B9%E0%A4%BE%E0%A4%97&amp;oldid=5634907</t>
   </si>
   <si>
     <t>भीमपलासी</t>
   </si>
   <si>
-    <t>Bhimpalasi</t>
-  </si>
-  <si>
-    <t>Hindustani classical raga</t>
-  </si>
-  <si>
-    <t>https://www.wikidata.org/wiki/Q45564</t>
-  </si>
-  <si>
-    <t>भूपाली</t>
-  </si>
-  <si>
-    <t>Bhoopali</t>
-  </si>
-  <si>
-    <t>https://www.wikidata.org/wiki/Q46954</t>
-  </si>
-  <si>
-    <t>बिहाग</t>
-  </si>
-  <si>
-    <t>Bihag</t>
-  </si>
-  <si>
-    <t>https://www.wikidata.org/wiki/Q4907048</t>
-  </si>
-  <si>
-    <t>दरबारी कान्हड़ा</t>
-  </si>
-  <si>
-    <t>Darbari Kanhada</t>
-  </si>
-  <si>
-    <t>Janya raga of Carnatic music, also used in Hindustani classical music</t>
-  </si>
-  <si>
-    <t>जन्य राग</t>
-  </si>
-  <si>
-    <t>https://www.wikidata.org/wiki/Q15681261</t>
-  </si>
-  <si>
-    <t>देश</t>
-  </si>
-  <si>
-    <t>Desh</t>
-  </si>
-  <si>
-    <t>https://www.wikidata.org/wiki/Q12434145</t>
-  </si>
-  <si>
-    <t>दुर्गा</t>
-  </si>
-  <si>
-    <t>Durga</t>
-  </si>
-  <si>
-    <t>https://www.wikidata.org/wiki/Q5316371</t>
-  </si>
-  <si>
-    <t>हमीर</t>
-  </si>
-  <si>
-    <t>Hameer</t>
-  </si>
-  <si>
-    <t>https://www.wikidata.org/wiki/Q5644481</t>
-  </si>
-  <si>
-    <t>काफ़ी</t>
-  </si>
-  <si>
-    <t>Kafi (raga)</t>
-  </si>
-  <si>
-    <t>https://www.wikidata.org/wiki/Q2560197</t>
-  </si>
-  <si>
-    <t>केदार</t>
-  </si>
-  <si>
-    <t>Kedar</t>
-  </si>
-  <si>
-    <t>https://www.wikidata.org/wiki/Q12420571</t>
-  </si>
-  <si>
-    <t>खमाज</t>
-  </si>
-  <si>
-    <t>Khamaj</t>
-  </si>
-  <si>
-    <t>https://www.wikidata.org/wiki/Q6399897</t>
-  </si>
-  <si>
-    <t>मालकौंस</t>
-  </si>
-  <si>
-    <t>Malkauns</t>
-  </si>
-  <si>
-    <t>https://www.wikidata.org/wiki/Q7377646</t>
-  </si>
-  <si>
-    <t>मुल्तानी</t>
-  </si>
-  <si>
-    <t>Multani</t>
-  </si>
-  <si>
-    <t>https://www.wikidata.org/wiki/Q6934367</t>
-  </si>
-  <si>
-    <t>पूरिया</t>
-  </si>
-  <si>
-    <t>Puriya</t>
-  </si>
-  <si>
-    <t>https://www.wikidata.org/wiki/Q7261299</t>
-  </si>
-  <si>
-    <t>पूरिया धनाश्री</t>
-  </si>
-  <si>
-    <t>Puriya Dhanashree</t>
-  </si>
-  <si>
-    <t>https://www.wikidata.org/wiki/Q7261302</t>
-  </si>
-  <si>
-    <t>तोड़ी</t>
-  </si>
-  <si>
-    <t>Todi</t>
-  </si>
-  <si>
-    <t>https://www.wikidata.org/wiki/Q7812775</t>
-  </si>
-  <si>
-    <t>यमन</t>
-  </si>
-  <si>
-    <t>Yaman</t>
-  </si>
-  <si>
-    <t>https://www.wikidata.org/wiki/Q8047871</t>
+    <t>यह राग काफी थाट से निकलता है। आरोह में रे और ध"' नहीं लगता और अवरोह में सब स्वर लगते हैं, इसलिये इस की जाति औडव-सम्पूर्ण मानी जाती है। इसमें ग"' और नी"' कोमल लगते हैं। वादी स्वर म"' और सम्वादी स्वर स"' माना जाता है।</t>
+  </si>
+  <si>
+    <t>https://hi.wikipedia.org/w/index.php?title=%E0%A4%AD%E0%A5%80%E0%A4%AE%E0%A4%AA%E0%A4%B2%E0%A4%BE%E0%A4%B8%E0%A5%80&amp;oldid=6287532</t>
+  </si>
+  <si>
+    <t>भैरव राग</t>
+  </si>
+  <si>
+    <t>भैरव राग राग भैरव थाट का राग है। यह राग भैरव थाट के नाम जैसे होने से इसे भैरव थाट का आश्रय राग कहा जाता है। इस राग में सात स्वर लगते हैं, इसलिये इसकी जाति सम्पूर्ण (सम्पूर्ण-सम्पूर्ण) मानी जाती है। इस राग में रे और ध स्वर कोमल लगते हैं जिसे इस प्रकार दर्शाया जाता है</t>
+  </si>
+  <si>
+    <t>https://hi.wikipedia.org/w/index.php?title=%E0%A4%AD%E0%A5%88%E0%A4%B0%E0%A4%B5_%E0%A4%B0%E0%A4%BE%E0%A4%97&amp;oldid=6383074</t>
+  </si>
+  <si>
+    <t>मल्हार राग</t>
+  </si>
+  <si>
+    <t>मल्हार राग/ मेघ मल्हार, हिंदुस्तानी व कर्नाटिक संगीत में पाया जाता है। मल्हार का मतलब बारिश या वर्षा है और माना जाता है कि मल्हार राग के गानों को गाने से वर्षा होता है। मल्हार राग को कर्नाटिक शैली में मधायामावती बुलाया जाता है। तानसेन और मीरा मल्हार राग में गाने गाने के लिए मशहूर थे। माना जाता है के तानसेन के 'मियाँ के मल्हार' गाने से सुखा ग्रस्त प्रदेश में भी बारिश होती थि। मल्हार राग के प्रसिद्द रचनाये : करे करे बदरा घटा घाना घोर घोर goor मियाँ की मल्हार</t>
+  </si>
+  <si>
+    <t>https://hi.wikipedia.org/w/index.php?title=%E0%A4%AE%E0%A4%B2%E0%A5%8D%E0%A4%B9%E0%A4%BE%E0%A4%B0_%E0%A4%B0%E0%A4%BE%E0%A4%97&amp;oldid=5248251</t>
+  </si>
+  <si>
+    <t>मालकोश</t>
+  </si>
+  <si>
+    <t>यह राग भैरवी थाट से निकलता है। इसमें ऋषभ और पंचम स्वर नहीं लगते इसलिये इसकी जाति औडव मानी जाती है। इसमें गंधार धैवत और निषाद कोमल लगते है। इसका वादी स्वर मध्यम तथा सम्वादी स्वर षड्ज माना जाता है।</t>
+  </si>
+  <si>
+    <t>https://hi.wikipedia.org/w/index.php?title=%E0%A4%AE%E0%A4%BE%E0%A4%B2%E0%A4%95%E0%A5%8B%E0%A4%B6&amp;oldid=3990180</t>
+  </si>
+  <si>
+    <t>राग अंजनी टोड़ी</t>
+  </si>
+  <si>
+    <t>राग अंजनी तोड़ी हिंदुस्तानी संगीत में एक राग है, जो किसी गीत के बीच में पंचम और मध्यम को जोड़ता है।</t>
+  </si>
+  <si>
+    <t>https://hi.wikipedia.org/w/index.php?title=%E0%A4%B0%E0%A4%BE%E0%A4%97_%E0%A4%85%E0%A4%82%E0%A4%9C%E0%A4%A8%E0%A5%80_%E0%A4%9F%E0%A5%8B%E0%A4%A1%E0%A4%BC%E0%A5%80&amp;oldid=6204776</t>
+  </si>
+  <si>
+    <t>राग गौड़सारङ्ग</t>
+  </si>
+  <si>
+    <t>गौड़ सारंग , भारतीय संगीत का एक राग है। इसके गायन का समय दोपहर (मध्याह्न काल) है।</t>
+  </si>
+  <si>
+    <t>https://hi.wikipedia.org/w/index.php?title=%E0%A4%B0%E0%A4%BE%E0%A4%97_%E0%A4%97%E0%A5%8C%E0%A4%A1%E0%A4%BC%E0%A4%B8%E0%A4%BE%E0%A4%B0%E0%A4%99%E0%A5%8D%E0%A4%97&amp;oldid=4789996</t>
+  </si>
+  <si>
+    <t>राग दरबारी कान्हड़ा</t>
+  </si>
+  <si>
+    <t>प्राचीन संगीत ग्रन्थों में राग दरबारी कान्हड़ा के लिये भिन्न नामों का उल्लेख मिलता है। कुछ ग्रन्थों में इसका नाम कणार्ट, कुछ में कणार्टकी तो अन्य ग्रन्थों में कणार्ट गौड़ उपलब्ध है। वस्तुत: कन्हण शब्द कणार्ट शब्द का ही अपभ्रंश रूप है। कान्हड़ा के पूर्व दरबारी शब्द का प्रयोग मुगल शासन के समय से प्रचलित हुआ ऐसा माना जाता है। कान्हड़ा के कुल कुल 18 प्रकार माने जाते हैं-</t>
+  </si>
+  <si>
+    <t>https://hi.wikipedia.org/w/index.php?title=%E0%A4%B0%E0%A4%BE%E0%A4%97_%E0%A4%A6%E0%A4%B0%E0%A4%AC%E0%A4%BE%E0%A4%B0%E0%A5%80_%E0%A4%95%E0%A4%BE%E0%A4%A8%E0%A5%8D%E0%A4%B9%E0%A4%A1%E0%A4%BC%E0%A4%BE&amp;oldid=5541652</t>
+  </si>
+  <si>
+    <t>राग बसंत</t>
+  </si>
+  <si>
+    <t>राग बसंत या राग वसंत शास्त्रीय संगीत की हिंदुस्तानी पद्धति का राग है। वसंत का अर्थ वसंत ऋतु से है, अतः इसे विशेष रूप से वसंत ऋतु में गाया बजाया जाता है। इसके आरोह में पाँच तथा अवरोह में सात स्वर होते हैं। अतः यह औडव-संपूर्ण जाति का राग है। वसंत ऋतु में गाया जाने के कारण इस राग में होलियाँ बहुत मिलती हैं। यह प्रसन्नता तथा उत्फुल्लता का राग है। ऐसा माना जाता है कि इसके गाने व सुनने से मन प्रसन्न हो जाता है। इसका गायन समय रात का अंतिम प्रहर है किंतु यह दिन या रात में किसी समय भी गाया बजाया जा सकता है। रागमाला में इसे राग हिंडोल का पुत्र माना गया है। यह पूर्वी थाट का राग है। शास्त्रों में इससे मिलते जुलते एक राग वसंत हिंडोल का उल्लेख भी मिलता है। यह एक अत्यंत प्राचीन राग है जिसका उल्लेख अनेक प्राचीन ग्रंथों में मिलता है।</t>
+  </si>
+  <si>
+    <t>https://hi.wikipedia.org/w/index.php?title=%E0%A4%B0%E0%A4%BE%E0%A4%97_%E0%A4%AC%E0%A4%B8%E0%A4%82%E0%A4%A4&amp;oldid=5196825</t>
+  </si>
+  <si>
+    <t>राग बहार</t>
+  </si>
+  <si>
+    <t>राग बहार काफ़ी थाट से उत्पन्न षाड़व षाड़व जाति का राग है। अर्थात इसके आरोह तथा अवरोह से छे छे स्वरों का प्रयोग होता है। इसके गाने का समय रात्रि का दूसरा प्रहर है। गांधार और निषाद दोनो स्वर कोमल है लेकिन गायक अक्सर दोनों निषाद लेते हैं, शुद्ध निषाद का प्रयोग मध्य सप्तक में होता है और वह भी आरोह में। अन्य स्वर शुद्ध लगते हैं। कुछ गायक मध्यम के साथ विवादी के रूप में शुद्ध गंधार का भी थोड़ा सा प्रयोग करते हैं। लेकिन यह नियम नहीं, इसके अवरोह में कभी कभी ऋषभ और धैवत दोनो वर्जित करते हुए निधनिप ऐसा प्रयोग होता है पर यह आवश्यक नहीं। आरोह में गमपगमधनिसां इस प्रकार पंचम का वक्र प्रयोग भी होता है जिससे रागरंजकता बढ़ती है। इस राग का वादी स्वर षडज तथा संवादी स्वर मध्यम हैं। राग विस्तार मध्य व तार सप्तक में होने के कारण यह चंचल प्रकृति का राग माना जाता है। मपगम धनिसां इसकी मुख्य पकड़ है। यह राग बाकी अनेक रागों के साथ मिलाकर भी गाया जाता हैं। जिस राग के साथ उसे मिश्रित किया जाता है उसे उस राग के साथ संयुक्त नाम से जाना जाता है। उदाहरण के लिए बागेश्री राग में इसे मिश्र करने से बागेश्री-बहार, वसंत-बहार, भैरव-बहार इत्यादि। परंतु मिश्रण का एक नियम हे कि जिसमें बहार मिश्र किया जाय वह राग शुद्ध मध्यम या पंचम में होना चाहिए क्योंकि बहार का मिश्रण शुद्ध मध्यम से ही शुरू होता है।</t>
+  </si>
+  <si>
+    <t>https://hi.wikipedia.org/w/index.php?title=%E0%A4%B0%E0%A4%BE%E0%A4%97_%E0%A4%AC%E0%A4%B9%E0%A4%BE%E0%A4%B0&amp;oldid=5425779</t>
+  </si>
+  <si>
+    <t>राग बागेश्वरी</t>
+  </si>
+  <si>
+    <t>राग बागेश्वरी काफी थाट का राग है इसके गायन वादन का समय रात्रि का है। इस राग मैं ७ स्वरो का प्रयोग हुआ है। गन्धार व निषाद कोमल है।</t>
+  </si>
+  <si>
+    <t>https://hi.wikipedia.org/w/index.php?title=%E0%A4%B0%E0%A4%BE%E0%A4%97_%E0%A4%AC%E0%A4%BE%E0%A4%97%E0%A5%87%E0%A4%B6%E0%A5%8D%E0%A4%B5%E0%A4%B0%E0%A5%80&amp;oldid=3071360</t>
+  </si>
+  <si>
+    <t>राग भूपाली</t>
+  </si>
+  <si>
+    <t>इस राग का चलन मुख्यत: मन्द्र और मध्य सप्तक के प्रतह्म हिस्से में होती है (पूर्वांग प्रधान राग)। इस राग में ठुमरी नहीं गायी जाती मगर, बड़ा खयाल, छोटा खयाल, तराना आदि गाया जाता है। कर्नाटक संगीत में इसे मोहन राग कहते हैं।</t>
+  </si>
+  <si>
+    <t>https://hi.wikipedia.org/w/index.php?title=%E0%A4%B0%E0%A4%BE%E0%A4%97_%E0%A4%AD%E0%A5%82%E0%A4%AA%E0%A4%BE%E0%A4%B2%E0%A5%80&amp;oldid=6252227</t>
+  </si>
+  <si>
+    <t>राग भैरवी</t>
+  </si>
+  <si>
+    <t>'''' रे ग ध नि कोमल राखत, मानत मध्यम वादी।</t>
+  </si>
+  <si>
+    <t>https://hi.wikipedia.org/w/index.php?title=%E0%A4%B0%E0%A4%BE%E0%A4%97_%E0%A4%AD%E0%A5%88%E0%A4%B0%E0%A4%B5%E0%A5%80&amp;oldid=5196824</t>
+  </si>
+  <si>
+    <t>राग मुल्ताली</t>
+  </si>
+  <si>
+    <t>थाठ: तोड़ी वादी: प संवादी : सा जाति : औडव-संपूर्ण आरोह में रे और ध वर्जित स्वर हैं गायन समय: दिन का चौथा प्रहर स्वर :- कोमल रे, कोमल ग, तीव्र म का प्रयोग, बाकी सब स्वर शुद्ध</t>
+  </si>
+  <si>
+    <t>https://hi.wikipedia.org/w/index.php?title=%E0%A4%B0%E0%A4%BE%E0%A4%97_%E0%A4%AE%E0%A5%81%E0%A4%B2%E0%A5%8D%E0%A4%A4%E0%A4%BE%E0%A4%B2%E0%A5%80&amp;oldid=5182492</t>
+  </si>
+  <si>
+    <t>राग मेघमल्लार</t>
+  </si>
+  <si>
+    <t>वर्षा ऋतु में गाने वाला राग, जिनसे बारिश होती है।</t>
+  </si>
+  <si>
+    <t>https://hi.wikipedia.org/w/index.php?title=%E0%A4%B0%E0%A4%BE%E0%A4%97_%E0%A4%AE%E0%A5%87%E0%A4%98%E0%A4%AE%E0%A4%B2%E0%A5%8D%E0%A4%B2%E0%A4%BE%E0%A4%B0&amp;oldid=6166770</t>
+  </si>
+  <si>
+    <t>राग ललित</t>
+  </si>
+  <si>
+    <t>राग बसंत या राग वसंत शास्त्रीय संगीत की हिंदुस्तानी पद्धति का राग है। राग ललित सन्धिप्रकाश रागो के अन्तर्गत आता है। यह एक गम्भी्र प्रकृति का उत्तरांग प्रधान राग है। इसे गाते व बजाते समय इसका विस्तार मन्द्र व मध्य सप्तकों में अधिक होता है। राग ललित दो मतों से गाया जाता है शुद्ध धैवत व कोमल धैवत परन्तु शु्द्ध धैवत से यह राग अधिक प्रचार में है।</t>
+  </si>
+  <si>
+    <t>https://hi.wikipedia.org/w/index.php?title=%E0%A4%B0%E0%A4%BE%E0%A4%97_%E0%A4%B2%E0%A4%B2%E0%A4%BF%E0%A4%A4&amp;oldid=6526615</t>
+  </si>
+  <si>
+    <t>राग सिंधुरा</t>
+  </si>
+  <si>
+    <t>राग सिंधुरा एक चंचल प्रकृति का राग है। यह की राग काफी के बहुत निकट है। राग काफी से इसे अलग दर्शाने के लिए कभी कभी निषाद शुद्ध का प्रयोग आरोह में इस तरह से किया जाता है - म प नि नि सा'। राग काफी में म प ग१ रे यह स्वर समूह राग वाचक है जबकि सिंधुरा में म प ; म ग१ रे ; म ग१ रे सा इस तरह से लिया जाता है।</t>
+  </si>
+  <si>
+    <t>https://hi.wikipedia.org/w/index.php?title=%E0%A4%B0%E0%A4%BE%E0%A4%97_%E0%A4%B8%E0%A4%BF%E0%A4%82%E0%A4%A7%E0%A5%81%E0%A4%B0%E0%A4%BE&amp;oldid=4920943</t>
+  </si>
+  <si>
+    <t>राग हंसध्वनि</t>
+  </si>
+  <si>
+    <t>राग हंसध्वनि कनार्टक पद्धति का एक राग है जो आजकल उत्तर भारत मे भी काफी प्रचलित है। इसके थाट के विषय में दो मत हैं कुछ विद्वान इसे बिलावल थाट तो कुछ कल्याण थाट जन्य भी मानते हैं। इस राग में मध्यम तथा धैवत स्वर वर्जित हैं अत: इसकी जाति औडव-औडव मानी जाती है। सभी शुद्ध स्वरों के प्रयोग के साथ ही पंचम रिषभ, रिषभ निषाद एवम षडज पंचम की स्वर संगतियाँ बार बार प्रयुक्त होती हैं। इसके निकट के रागो में राग शंकरा का नाम लिया जाता है। गायन समय रात्रि का द्वितीय प्रहर है।</t>
+  </si>
+  <si>
+    <t>https://hi.wikipedia.org/w/index.php?title=%E0%A4%B0%E0%A4%BE%E0%A4%97_%E0%A4%B9%E0%A4%82%E0%A4%B8%E0%A4%A7%E0%A5%8D%E0%A4%B5%E0%A4%A8%E0%A4%BF&amp;oldid=6094654</t>
+  </si>
+  <si>
+    <t>राग हिंडोल</t>
+  </si>
+  <si>
+    <t>राग हिंडोल या राग हिंदोल का जन्म कल्याण थाट से माना गया है। इसमें मध्यम तीव्र तथा निषाद व गंधार कोमल लगते हैं। ऋषभ तथा पंचम वर्जित है। इसकी जाति ओड़व ओड़व है तथा वादी स्वर धैवत व संवादी स्वर गांधार है। गायन का समय प्रातःकाल है। शुद्ध निषाद, रिषभ और पंचम इस स्वर इसमें वर्ज्य हैं। तीव्र मध्यम वाला यह एक ही राग है जिसको प्रातःकाल गाया जाता है। अन्य सभी तीव्र मध्यम वाले रागों का गायन समय रात्रि में होता है।</t>
+  </si>
+  <si>
+    <t>https://hi.wikipedia.org/w/index.php?title=%E0%A4%B0%E0%A4%BE%E0%A4%97_%E0%A4%B9%E0%A4%BF%E0%A4%82%E0%A4%A1%E0%A5%8B%E0%A4%B2&amp;oldid=5425780</t>
+  </si>
+  <si>
+    <t>केदार राग</t>
+  </si>
+  <si>
+    <t>यह राग कल्याण थाट से निकलता है। इसमें शुद्ध व तीव्र दोनों म लगाये जाते है। इसके आरोह में रे और ग को नहीं लगाते और अवरोह में ग नहीं लगाते इसलिये इसकी जाति औडव-षाड़व मानी जाती है। वादी स्वर म और संवादी स्वर सा माना जाता है।</t>
+  </si>
+  <si>
+    <t>https://hi.wikipedia.org/w/index.php?title=%E0%A4%95%E0%A5%87%E0%A4%A6%E0%A4%BE%E0%A4%B0_%E0%A4%B0%E0%A4%BE%E0%A4%97&amp;oldid=4876400</t>
+  </si>
+  <si>
+    <t>आशवरी</t>
+  </si>
+  <si>
+    <t>आसावरी ( या, आसावरी) प्राचीन भारतीय संगीताचार्यों के अनुसार राग 'श्री' की एक प्रमुख रागिनी। ऋतु, समय और भावादि का वैज्ञानिक विश्लेषण करके प्रमुख 132 प्रकार के राग-रागिनियों की कल्पना की गई थी किंतु आधुनिक विद्वानों ने यह विभेद हटाकर सबको राग की ही संज्ञा दी है। आशावरी वियोगशृंगार की रागिनी (राग) है और इसके गायन का समय दिन का द्वितीय प्रहर है। इसका लक्षण ' रागप्रकाशिका ' नामक ग्रंथ (सन्‌ 1899 ई.) में यों दिया है:</t>
+  </si>
+  <si>
+    <t>https://hi.wikipedia.org/w/index.php?title=%E0%A4%86%E0%A4%B6%E0%A4%B5%E0%A4%B0%E0%A5%80&amp;oldid=4817759</t>
   </si>
 </sst>
 </file>
@@ -238,10 +289,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -582,17 +636,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="27" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="13" customWidth="1"/>
+    <col min="1" max="1" width="36" customWidth="1"/>
+    <col min="2" max="2" width="110" customWidth="1"/>
+    <col min="3" max="3" width="90" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -602,304 +654,284 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+    </row>
+    <row r="2" ht="48" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="C2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="3" ht="48" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" t="s">
+      <c r="C3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" t="s">
+    </row>
+    <row r="4" ht="48" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C3" t="s">
+    </row>
+    <row r="5" ht="64" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="B5" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="C5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B4" t="s">
+    </row>
+    <row r="6" ht="64" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="B6" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="C6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B5" t="s">
+    </row>
+    <row r="7" ht="48" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" t="s">
+      <c r="B7" s="2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="C7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B6" t="s">
+    </row>
+    <row r="8" ht="48" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C6" t="s">
+      <c r="B8" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D6" t="s">
+      <c r="C8" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E6" t="s">
+    </row>
+    <row r="9" ht="80" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="B9" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C9" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" t="s">
+    </row>
+    <row r="10" ht="48" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="B10" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C10" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" t="s">
-        <v>8</v>
-      </c>
-      <c r="E8" t="s">
+    </row>
+    <row r="11" ht="48" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="B11" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C11" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E9" t="s">
+    </row>
+    <row r="12" ht="48" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="B12" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C12" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D10" t="s">
-        <v>8</v>
-      </c>
-      <c r="E10" t="s">
+    </row>
+    <row r="13" ht="64" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="B13" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C13" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D11" t="s">
-        <v>8</v>
-      </c>
-      <c r="E11" t="s">
+    </row>
+    <row r="14" ht="128" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="B14" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C14" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C12" t="s">
-        <v>12</v>
-      </c>
-      <c r="D12" t="s">
-        <v>8</v>
-      </c>
-      <c r="E12" t="s">
+    </row>
+    <row r="15" ht="208" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="B15" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C15" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C13" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" t="s">
-        <v>8</v>
-      </c>
-      <c r="E13" t="s">
+    </row>
+    <row r="16" ht="42" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+      <c r="B16" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C16" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C14" t="s">
-        <v>12</v>
-      </c>
-      <c r="D14" t="s">
-        <v>8</v>
-      </c>
-      <c r="E14" t="s">
+    </row>
+    <row r="17" ht="48" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+      <c r="B17" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C17" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C15" t="s">
-        <v>7</v>
-      </c>
-      <c r="D15" t="s">
-        <v>8</v>
-      </c>
-      <c r="E15" t="s">
+    </row>
+    <row r="18" ht="42" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="B18" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C18" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C16" t="s">
-        <v>7</v>
-      </c>
-      <c r="D16" t="s">
-        <v>8</v>
-      </c>
-      <c r="E16" t="s">
+    </row>
+    <row r="19" ht="42" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+      <c r="B19" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C19" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C17" t="s">
-        <v>7</v>
-      </c>
-      <c r="D17" t="s">
-        <v>8</v>
-      </c>
-      <c r="E17" t="s">
+    </row>
+    <row r="20" ht="42" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+      <c r="B20" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C20" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C18" t="s">
-        <v>7</v>
-      </c>
-      <c r="D18" t="s">
-        <v>8</v>
-      </c>
-      <c r="E18" t="s">
+    </row>
+    <row r="21" ht="64" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
         <v>60</v>
       </c>
+      <c r="B21" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="22" ht="64" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="23" ht="80" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="24" ht="80" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="25" ht="48" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="26" ht="80" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>77</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E1"/>
+  <autoFilter ref="A1:C1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>